<commit_message>
Renomeia campo Cidade/Bairro para Endereço em clientes
</commit_message>
<xml_diff>
--- a/public/modelos/modelo-clientes.xlsx
+++ b/public/modelos/modelo-clientes.xlsx
@@ -19,7 +19,7 @@
     <t>Tipo Cliente</t>
   </si>
   <si>
-    <t>Cidade ou Bairro</t>
+    <t>Endereço</t>
   </si>
   <si>
     <t>Telefone</t>
@@ -31,7 +31,7 @@
     <t>Buffet</t>
   </si>
   <si>
-    <t>Centro</t>
+    <t>Rua das Flores, 123 - Centro, São Paulo/SP</t>
   </si>
   <si>
     <t>(11) 91234-5678</t>
@@ -43,7 +43,7 @@
     <t>Pessoa Física</t>
   </si>
   <si>
-    <t>Jardim das Flores</t>
+    <t>Av. Paulista, 900, apto 45 - Bela Vista, São Paulo/SP</t>
   </si>
   <si>
     <t>(11) 98888-1234</t>

</xml_diff>